<commit_message>
Update optimized dataset and add temporary file. Commented out checkpoint code as not needed for small datasets.
</commit_message>
<xml_diff>
--- a/Datasets/dsm_optimize_for_consolidation_clean_optimized.xlsx
+++ b/Datasets/dsm_optimize_for_consolidation_clean_optimized.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dsm" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="grouping" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="consolidation" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="dsm" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="grouping" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="consolidation" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -40,12 +40,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00800026"/>
+        <fgColor rgb="00FFFFCC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFCC"/>
+        <fgColor rgb="00800026"/>
       </patternFill>
     </fill>
   </fills>
@@ -655,10 +655,10 @@
         <v>1</v>
       </c>
       <c r="H6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -689,10 +689,10 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -717,10 +717,10 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
         <v>0</v>
@@ -751,10 +751,10 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>1</v>
@@ -832,7 +832,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Unit 1</t>
+          <t>Unit 0</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Unit 1</t>
+          <t>Unit 0</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -862,7 +862,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Unit 1</t>
+          <t>Unit 0</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -877,7 +877,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Unit 1</t>
+          <t>Unit 0</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -892,7 +892,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Unit 1</t>
+          <t>Unit 0</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Unit 1</t>
+          <t>Unit 0</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">

</xml_diff>